<commit_message>
fix: resolve MaxListenersExceededWarning on ServerResponse and add setup_and_run.sh
</commit_message>
<xml_diff>
--- a/demo_sample.xlsx
+++ b/demo_sample.xlsx
@@ -1,14 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1086D82-2A55-45F6-8B21-12E87C7CDC4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-28800" yWindow="2415" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Danh sách mẫu" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Danh sách mẫu" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -35,18 +31,30 @@
     <t>Sách: A Light in the Attic</t>
   </si>
   <si>
+    <t>https://books.toscrape.com/catalogue/a-light-in-the-attic_1000/index.html</t>
+  </si>
+  <si>
     <t>Thử selector: h1 hoặc .price_color</t>
   </si>
   <si>
     <t>Sách: Tipping the Velvet</t>
   </si>
   <si>
+    <t>https://books.toscrape.com/catalogue/tipping-the-velvet_999/index.html</t>
+  </si>
+  <si>
     <t>Sách: Soumission</t>
   </si>
   <si>
+    <t>https://books.toscrape.com/catalogue/soumission_998/index.html</t>
+  </si>
+  <si>
     <t>Wikipedia: Next.js</t>
   </si>
   <si>
+    <t>https://en.wikipedia.org/wiki/Next.js</t>
+  </si>
+  <si>
     <t>Thử selector: h1#firstHeading, h1</t>
   </si>
   <si>
@@ -63,45 +71,24 @@
   </si>
   <si>
     <t>Thử selector: .quote .text, h1 a</t>
-  </si>
-  <si>
-    <t>https://giftee-na2.e-gift.co/c/f7h7p2YwkfeuC1Va/1</t>
-  </si>
-  <si>
-    <t>https://giftee-na2.e-gift.co/c/Rb9QDRW6Rccufj9x/1</t>
-  </si>
-  <si>
-    <t>https://giftee-na2.e-gift.co/c/6xzqcRkce1wDdSzo/1</t>
-  </si>
-  <si>
-    <t>https://giftee-na2.e-gift.co/c/Rcd3S2ctb4A5Rrnu/1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -126,11 +113,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -138,12 +124,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -480,9 +462,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -490,7 +472,7 @@
     <col min="4" max="5" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" ht="28" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -507,98 +489,98 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>16</v>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>19</v>
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>15</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="E7" s="2"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{829741BA-6839-422E-AEF8-6D6405DBB00D}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{58AEC894-2F0C-45AF-9E54-2463D441478D}"/>
-    <hyperlink ref="C4" r:id="rId3" xr:uid="{179D0350-EDDA-4906-A416-4C67310E5BC5}"/>
-    <hyperlink ref="C5" r:id="rId4" xr:uid="{16F9139E-3982-44F1-B8F7-4E9F8574BDFC}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update demo_sample.xlsx to reflect recent changes in data structure and content
</commit_message>
<xml_diff>
--- a/demo_sample.xlsx
+++ b/demo_sample.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCA0821B-89F1-43DB-8668-D66B88A05E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-28800" yWindow="2415" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Danh sách mẫu" state="visible" r:id="rId4"/>
+    <sheet name="Danh sách mẫu" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
     <t>STT</t>
   </si>
@@ -31,64 +35,64 @@
     <t>Sách: A Light in the Attic</t>
   </si>
   <si>
-    <t>https://books.toscrape.com/catalogue/a-light-in-the-attic_1000/index.html</t>
-  </si>
-  <si>
     <t>Thử selector: h1 hoặc .price_color</t>
   </si>
   <si>
     <t>Sách: Tipping the Velvet</t>
   </si>
   <si>
-    <t>https://books.toscrape.com/catalogue/tipping-the-velvet_999/index.html</t>
-  </si>
-  <si>
     <t>Sách: Soumission</t>
   </si>
   <si>
-    <t>https://books.toscrape.com/catalogue/soumission_998/index.html</t>
-  </si>
-  <si>
     <t>Wikipedia: Next.js</t>
   </si>
   <si>
-    <t>https://en.wikipedia.org/wiki/Next.js</t>
-  </si>
-  <si>
     <t>Thử selector: h1#firstHeading, h1</t>
   </si>
   <si>
     <t>Wikipedia: Web Scraping</t>
   </si>
   <si>
-    <t>https://en.wikipedia.org/wiki/Web_scraping</t>
-  </si>
-  <si>
-    <t>Quotes: Albert Einstein</t>
-  </si>
-  <si>
-    <t>https://quotes.toscrape.com/</t>
-  </si>
-  <si>
-    <t>Thử selector: .quote .text, h1 a</t>
+    <t>https://giftee-na2.e-gift.co/c/f7h7p2YwkfeuC1Va/1</t>
+  </si>
+  <si>
+    <t>https://giftee-na2.e-gift.co/c/Rb9QDRW6Rccufj9x/1</t>
+  </si>
+  <si>
+    <t>https://giftee-na2.e-gift.co/c/6xzqcRkce1wDdSzo/1</t>
+  </si>
+  <si>
+    <t>https://giftee-na2.e-gift.co/c/Rcd3S2ctb4A5Rrnu/1</t>
+  </si>
+  <si>
+    <t>https://giftee-na2.e-gift.co/c/X1K3hrg5D6psKVPy</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
+      <u/>
       <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -113,10 +117,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -124,8 +129,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -462,9 +471,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -472,7 +481,7 @@
     <col min="4" max="5" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -489,98 +498,85 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="2"/>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="2"/>
+        <v>6</v>
+      </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="2"/>
+        <v>6</v>
+      </c>
     </row>
-    <row r="5" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="2"/>
+        <v>10</v>
+      </c>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" s="2" customFormat="1" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="2"/>
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{240D00F6-4750-4429-92DD-3BB6D0BCAF50}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{B2532C33-8C76-47C3-B850-FBED5C3DE799}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{D9B1BCD5-7128-45AE-B584-00D5B57ED1E4}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{FA861D59-4AC3-4DBA-B3D6-04FF4B7E44FA}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{637E1227-CA7E-44E1-833F-3FA1A69B8A4B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>